<commit_message>
update error messages and fix tests
</commit_message>
<xml_diff>
--- a/backend/fms_core/tests/invalid_templates/Sample_Rename_v5_6_0_multiple_samples.xlsx
+++ b/backend/fms_core/tests/invalid_templates/Sample_Rename_v5_6_0_multiple_samples.xlsx
@@ -25,7 +25,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="A6" authorId="0">
+    <comment ref="A2" authorId="0">
       <text>
         <r>
           <rPr>
@@ -37,7 +37,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B6" authorId="0">
+    <comment ref="B2" authorId="0">
       <text>
         <r>
           <rPr>
@@ -49,7 +49,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C6" authorId="0">
+    <comment ref="C2" authorId="0">
       <text>
         <r>
           <rPr>
@@ -61,7 +61,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D6" authorId="0">
+    <comment ref="D2" authorId="0">
       <text>
         <r>
           <rPr>
@@ -73,7 +73,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E6" authorId="0">
+    <comment ref="E2" authorId="0">
       <text>
         <r>
           <rPr>
@@ -85,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F6" authorId="0">
+    <comment ref="F2" authorId="0">
       <text>
         <r>
           <rPr>
@@ -97,7 +97,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G6" authorId="0">
+    <comment ref="G2" authorId="0">
       <text>
         <r>
           <rPr>
@@ -114,21 +114,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">Sample Rename Template</t>
   </si>
   <si>
-    <t xml:space="preserve">Naming Rules</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Only use the following characters for Sample Name and Sample Alias: a-z, A-Z, 0-9, underscore (_), hyphen (-)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Container Barcode</t>
   </si>
   <si>
-    <t xml:space="preserve">Container Coordinate</t>
+    <t xml:space="preserve">Container Coordinates</t>
   </si>
   <si>
     <t xml:space="preserve">Index Name</t>
@@ -194,6 +188,7 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -201,24 +196,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD1D1D1"/>
-        <bgColor rgb="FFC0C0C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFA6A6"/>
-        <bgColor rgb="FFFFCC99"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -261,7 +244,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -274,15 +257,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -320,7 +295,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD1D1D1"/>
+      <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -334,7 +309,7 @@
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFFA6A6"/>
+      <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
@@ -538,7 +513,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="1" style="1" width="29.63"/>
@@ -549,62 +524,47 @@
         <v>0</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
+      <c r="D3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>